<commit_message>
Update Gantt planning and Trello tasks
</commit_message>
<xml_diff>
--- a/Gantt.xlsx
+++ b/Gantt.xlsx
@@ -2,11 +2,11 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Synthèse" sheetId="1" r:id="Rae176b3ca121446c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Gantt" sheetId="2" r:id="R14232e8d527242ef"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Suivi réel" sheetId="3" r:id="R41ec0b0d3f20441f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Trello" sheetId="4" r:id="R5ba6fea2dc78447f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Consignes" sheetId="5" r:id="Re35d04324b46440f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Synthèse" sheetId="1" r:id="R8dc9d68224284b79"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Gantt" sheetId="2" r:id="R9100f063915f4d13"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Suivi réel" sheetId="3" r:id="R01a520aeb3494c6e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Trello" sheetId="4" r:id="R332838df465a4e9f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Consignes" sheetId="5" r:id="R21b67844f78044b5"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1014,7 +1014,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Rac95e87dde3f4e57"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R0609bf6b0022452d"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -1071,7 +1071,7 @@
     <x:tableColumn id="5" name="Échéance"/>
     <x:tableColumn id="6" name="Label"/>
     <x:tableColumn id="7" name="Charge h/h"/>
-    <x:tableColumn id="8" name="Ajouté / source"/>
+    <x:tableColumn id="8" name="Pourquoi c'est là"/>
   </x:tableColumns>
   <x:tableStyleInfo name="TableStyleMedium2" showRowStripes="1"/>
 </x:table>
@@ -1637,7 +1637,7 @@
     <x:mergeCell ref="A30:H33"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8255418738bb44af"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf0ad1629022145b5"/>
 </x:worksheet>
 </file>
 
@@ -3318,7 +3318,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7cf0df09a88f4da4"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R503eb1aa5563446d"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4448,7 +4448,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf322e74602754545"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb4a772165c294f2c"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4469,28 +4469,28 @@
   <x:sheetData>
     <x:row r="1" ht="25.5" customHeight="1">
       <x:c r="A1" s="4" t="str">
-        <x:v>Cartes Trello prêtes à copier</x:v>
+        <x:v>Cartes Trello - version claire et dynamique</x:v>
       </x:c>
       <x:c r="B1" s="4" t="str">
-        <x:v>Cartes Trello prêtes à copier</x:v>
+        <x:v>Cartes Trello - version claire et dynamique</x:v>
       </x:c>
       <x:c r="C1" s="4" t="str">
-        <x:v>Cartes Trello prêtes à copier</x:v>
+        <x:v>Cartes Trello - version claire et dynamique</x:v>
       </x:c>
       <x:c r="D1" s="4" t="str">
-        <x:v>Cartes Trello prêtes à copier</x:v>
+        <x:v>Cartes Trello - version claire et dynamique</x:v>
       </x:c>
       <x:c r="E1" s="4" t="str">
-        <x:v>Cartes Trello prêtes à copier</x:v>
+        <x:v>Cartes Trello - version claire et dynamique</x:v>
       </x:c>
       <x:c r="F1" s="4" t="str">
-        <x:v>Cartes Trello prêtes à copier</x:v>
+        <x:v>Cartes Trello - version claire et dynamique</x:v>
       </x:c>
       <x:c r="G1" s="4" t="str">
-        <x:v>Cartes Trello prêtes à copier</x:v>
+        <x:v>Cartes Trello - version claire et dynamique</x:v>
       </x:c>
       <x:c r="H1" s="4" t="str">
-        <x:v>Cartes Trello prêtes à copier</x:v>
+        <x:v>Cartes Trello - version claire et dynamique</x:v>
       </x:c>
     </x:row>
     <x:row r="3">
@@ -4516,7 +4516,7 @@
         <x:v>Charge h/h</x:v>
       </x:c>
       <x:c r="H3" s="21" t="str">
-        <x:v>Ajouté / source</x:v>
+        <x:v>Pourquoi c'est là</x:v>
       </x:c>
     </x:row>
     <x:row r="4" ht="81" customHeight="1">
@@ -4527,12 +4527,13 @@
         <x:v>Former l'équipe et définir les rôles</x:v>
       </x:c>
       <x:c r="C4" s="72" t="str">
-        <x:v>Objectif : Identifier les membres du groupe, répartir les responsabilités et clarifier le rôle de chacun.
-À vérifier :
-- Livrable produit : Rôles d'équipe
-- Carte tenue à jour dans la bonne colonne Trello
-- Contrôle consigne : Consigne Projet.pdf p.3
-Charge : 2 h/h | Échéance : 18.03.2026</x:v>
+        <x:v>Ce qu'on fait : Identifier les membres du groupe, répartir les responsabilités et clarifier le rôle de chacun.
+Done quand :
+- On a quelque chose de concret : Rôles d'équipe
+- La carte est dans la bonne colonne Trello
+- Ça respecte la consigne : Consigne Projet.pdf p.3
+Charge : 2 h/h
+Deadline : 18.03.2026</x:v>
       </x:c>
       <x:c r="D4" s="72" t="str">
         <x:v>Thierry, Dan, Jason</x:v>
@@ -4558,12 +4559,13 @@
         <x:v>Choisir le sujet Game Store et le faire valider</x:v>
       </x:c>
       <x:c r="C5" s="75" t="str">
-        <x:v>Objectif : Décrire le sujet, expliquer le choix et obtenir la validation de l'enseignant.
-À vérifier :
-- Livrable produit : Sujet validé
-- Carte tenue à jour dans la bonne colonne Trello
-- Contrôle consigne : Consigne Projet.pdf p.1
-Charge : 4 h/h | Échéance : 20.03.2026</x:v>
+        <x:v>Ce qu'on fait : Décrire le sujet, expliquer le choix et obtenir la validation de l'enseignant.
+Done quand :
+- On a quelque chose de concret : Sujet validé
+- La carte est dans la bonne colonne Trello
+- Ça respecte la consigne : Consigne Projet.pdf p.1
+Charge : 4 h/h
+Deadline : 20.03.2026</x:v>
       </x:c>
       <x:c r="D5" s="75" t="str">
         <x:v>Thierry, Dan, Jason</x:v>
@@ -4589,12 +4591,13 @@
         <x:v>Créer le tableau Trello et inviter l'enseignant</x:v>
       </x:c>
       <x:c r="C6" s="75" t="str">
-        <x:v>Objectif : Créer les colonnes minimales, inviter edu-sotoperafao@eduge.ch et vérifier que chaque tâche a un responsable.
-À vérifier :
-- Livrable produit : Tableau Trello prêt
-- Carte tenue à jour dans la bonne colonne Trello
-- Contrôle consigne : Consigne Projet.pdf p.2
-Charge : 2 h/h | Échéance : 20.03.2026</x:v>
+        <x:v>Ce qu'on fait : Créer les colonnes minimales, inviter edu-sotoperafao@eduge.ch et vérifier que chaque tâche a un responsable.
+Done quand :
+- On a quelque chose de concret : Tableau Trello prêt
+- La carte est dans la bonne colonne Trello
+- Ça respecte la consigne : Consigne Projet.pdf p.2
+Charge : 2 h/h
+Deadline : 20.03.2026</x:v>
       </x:c>
       <x:c r="D6" s="75" t="str">
         <x:v>Dan</x:v>
@@ -4620,12 +4623,13 @@
         <x:v>Définir le périmètre MVP et les objectifs</x:v>
       </x:c>
       <x:c r="C7" s="75" t="str">
-        <x:v>Objectif : Définir les fonctionnalités indispensables du site Game Store et les objectifs mesurables du projet.
-À vérifier :
-- Livrable produit : Objectifs MVP
-- Carte tenue à jour dans la bonne colonne Trello
-- Contrôle consigne : Consigne Projet.pdf p.3
-Charge : 4 h/h | Échéance : 21.03.2026</x:v>
+        <x:v>Ce qu'on fait : Définir les fonctionnalités indispensables du site Game Store et les objectifs mesurables du projet.
+Done quand :
+- On a quelque chose de concret : Objectifs MVP
+- La carte est dans la bonne colonne Trello
+- Ça respecte la consigne : Consigne Projet.pdf p.3
+Charge : 4 h/h
+Deadline : 21.03.2026</x:v>
       </x:c>
       <x:c r="D7" s="75" t="str">
         <x:v>Thierry, Dan, Jason</x:v>
@@ -4651,12 +4655,13 @@
         <x:v>Lister les tâches, estimations et responsables</x:v>
       </x:c>
       <x:c r="C8" s="75" t="str">
-        <x:v>Objectif : Créer la liste complète des tâches, avec description, responsable et estimation en heure/homme.
-À vérifier :
-- Livrable produit : Liste des tâches
-- Carte tenue à jour dans la bonne colonne Trello
-- Contrôle consigne : Consigne Projet.pdf p.3
-Charge : 6 h/h | Échéance : 24.03.2026</x:v>
+        <x:v>Ce qu'on fait : Créer la liste complète des tâches, avec description, responsable et estimation en heure/homme.
+Done quand :
+- On a quelque chose de concret : Liste des tâches
+- La carte est dans la bonne colonne Trello
+- Ça respecte la consigne : Consigne Projet.pdf p.3
+Charge : 6 h/h
+Deadline : 24.03.2026</x:v>
       </x:c>
       <x:c r="D8" s="75" t="str">
         <x:v>Thierry, Dan, Jason</x:v>
@@ -4682,12 +4687,13 @@
         <x:v>Produire le Gantt prévisionnel initial</x:v>
       </x:c>
       <x:c r="C9" s="75" t="str">
-        <x:v>Objectif : Construire le planning initial en Excel avec jalons et estimation heure/homme.
-À vérifier :
-- Livrable produit : Gantt initial
-- Carte tenue à jour dans la bonne colonne Trello
-- Contrôle consigne : Consigne Projet.pdf p.2-p.3
-Charge : 4 h/h | Échéance : 31.03.2026</x:v>
+        <x:v>Ce qu'on fait : Construire le planning initial en Excel avec jalons et estimation heure/homme.
+Done quand :
+- On a quelque chose de concret : Gantt initial
+- La carte est dans la bonne colonne Trello
+- Ça respecte la consigne : Consigne Projet.pdf p.2-p.3
+Charge : 4 h/h
+Deadline : 31.03.2026</x:v>
       </x:c>
       <x:c r="D9" s="75" t="str">
         <x:v>Thierry</x:v>
@@ -4713,12 +4719,13 @@
         <x:v>Rédiger la documentation v1 avec méthode des 6 étapes</x:v>
       </x:c>
       <x:c r="C10" s="75" t="str">
-        <x:v>Objectif : Rédiger description, choix, équipe, méthode des 6 étapes, liste des tâches et planification.
-À vérifier :
-- Livrable produit : Documentation v1
-- Carte tenue à jour dans la bonne colonne Trello
-- Contrôle consigne : Consigne Projet.pdf p.3
-Charge : 8 h/h | Échéance : 31.03.2026</x:v>
+        <x:v>Ce qu'on fait : Rédiger description, choix, équipe, méthode des 6 étapes, liste des tâches et planification.
+Done quand :
+- On a quelque chose de concret : Documentation v1
+- La carte est dans la bonne colonne Trello
+- Ça respecte la consigne : Consigne Projet.pdf p.3
+Charge : 8 h/h
+Deadline : 31.03.2026</x:v>
       </x:c>
       <x:c r="D10" s="75" t="str">
         <x:v>Jason</x:v>
@@ -4744,11 +4751,12 @@
         <x:v>Définir l'architecture du site et les parcours utilisateurs</x:v>
       </x:c>
       <x:c r="C11" s="75" t="str">
-        <x:v>Objectif : Prévoir navigation, pages principales, parcours consultation, inscription, connexion et profil.
-À vérifier :
-- Livrable produit : Architecture fonctionnelle
-- Carte tenue à jour dans la bonne colonne Trello
-Charge : 6 h/h | Échéance : 04.04.2026</x:v>
+        <x:v>Ce qu'on fait : Prévoir navigation, pages principales, parcours consultation, inscription, connexion et profil.
+Done quand :
+- On a quelque chose de concret : Architecture fonctionnelle
+- La carte est dans la bonne colonne Trello
+Charge : 6 h/h
+Deadline : 04.04.2026</x:v>
       </x:c>
       <x:c r="D11" s="75" t="str">
         <x:v>Thierry, Dan, Jason</x:v>
@@ -4774,11 +4782,12 @@
         <x:v>Mettre en place le repo, Docker, Apache, PHP et MySQL</x:v>
       </x:c>
       <x:c r="C12" s="75" t="str">
-        <x:v>Objectif : Préparer Dockerfile, docker-compose, serveur web PHP et base MySQL pour un lancement local simple.
-À vérifier :
-- Livrable produit : Docker fonctionnel
-- Carte tenue à jour dans la bonne colonne Trello
-Charge : 8 h/h | Échéance : 07.04.2026</x:v>
+        <x:v>Ce qu'on fait : Préparer Dockerfile, docker-compose, serveur web PHP et base MySQL pour un lancement local simple.
+Done quand :
+- On a quelque chose de concret : Docker fonctionnel
+- La carte est dans la bonne colonne Trello
+Charge : 8 h/h
+Deadline : 07.04.2026</x:v>
       </x:c>
       <x:c r="D12" s="75" t="str">
         <x:v>Thierry</x:v>
@@ -4804,11 +4813,12 @@
         <x:v>Créer le modèle de données et le script SQL</x:v>
       </x:c>
       <x:c r="C13" s="75" t="str">
-        <x:v>Objectif : Définir les tables utiles au site, écrire schema.sql et documenter les choix de modélisation.
-À vérifier :
-- Livrable produit : Schema SQL
-- Carte tenue à jour dans la bonne colonne Trello
-Charge : 8 h/h | Échéance : 08.04.2026</x:v>
+        <x:v>Ce qu'on fait : Définir les tables utiles au site, écrire schema.sql et documenter les choix de modélisation.
+Done quand :
+- On a quelque chose de concret : Schema SQL
+- La carte est dans la bonne colonne Trello
+Charge : 8 h/h
+Deadline : 08.04.2026</x:v>
       </x:c>
       <x:c r="D13" s="75" t="str">
         <x:v>Dan</x:v>
@@ -4834,11 +4844,12 @@
         <x:v>Créer les pages HTML principales</x:v>
       </x:c>
       <x:c r="C14" s="75" t="str">
-        <x:v>Objectif : Réaliser accueil, à propos, avis, jeux, profil, inscription, connexion et pages de résultat.
-À vérifier :
-- Livrable produit : Pages principales
-- Carte tenue à jour dans la bonne colonne Trello
-Charge : 16 h/h | Échéance : 15.04.2026</x:v>
+        <x:v>Ce qu'on fait : Réaliser accueil, à propos, avis, jeux, profil, inscription, connexion et pages de résultat.
+Done quand :
+- On a quelque chose de concret : Pages principales
+- La carte est dans la bonne colonne Trello
+Charge : 16 h/h
+Deadline : 15.04.2026</x:v>
       </x:c>
       <x:c r="D14" s="75" t="str">
         <x:v>Jason</x:v>
@@ -4864,11 +4875,12 @@
         <x:v>Construire le catalogue de jeux et les fiches détaillées</x:v>
       </x:c>
       <x:c r="C15" s="75" t="str">
-        <x:v>Objectif : Renseigner les jeux, prix, dates, images, descriptions et navigation vers les fiches.
-À vérifier :
-- Livrable produit : Catalogue jeux
-- Carte tenue à jour dans la bonne colonne Trello
-Charge : 12 h/h | Échéance : 18.04.2026</x:v>
+        <x:v>Ce qu'on fait : Renseigner les jeux, prix, dates, images, descriptions et navigation vers les fiches.
+Done quand :
+- On a quelque chose de concret : Catalogue jeux
+- La carte est dans la bonne colonne Trello
+Charge : 12 h/h
+Deadline : 18.04.2026</x:v>
       </x:c>
       <x:c r="D15" s="75" t="str">
         <x:v>Thierry</x:v>
@@ -4894,11 +4906,12 @@
         <x:v>Ajouter recherche, suggestions et navigation cartes</x:v>
       </x:c>
       <x:c r="C16" s="75" t="str">
-        <x:v>Objectif : Brancher la barre de recherche, les suggestions et la navigation depuis les cartes de jeux.
-À vérifier :
-- Livrable produit : Recherche fonctionnelle
-- Carte tenue à jour dans la bonne colonne Trello
-Charge : 8 h/h | Échéance : 18.04.2026</x:v>
+        <x:v>Ce qu'on fait : Brancher la barre de recherche, les suggestions et la navigation depuis les cartes de jeux.
+Done quand :
+- On a quelque chose de concret : Recherche fonctionnelle
+- La carte est dans la bonne colonne Trello
+Charge : 8 h/h
+Deadline : 18.04.2026</x:v>
       </x:c>
       <x:c r="D16" s="75" t="str">
         <x:v>Dan</x:v>
@@ -4924,11 +4937,12 @@
         <x:v>Harmoniser le CSS et le responsive</x:v>
       </x:c>
       <x:c r="C17" s="75" t="str">
-        <x:v>Objectif : Rendre les pages cohérentes visuellement et vérifier l'affichage desktop/mobile.
-À vérifier :
-- Livrable produit : Style homogène
-- Carte tenue à jour dans la bonne colonne Trello
-Charge : 12 h/h | Échéance : 18.04.2026</x:v>
+        <x:v>Ce qu'on fait : Rendre les pages cohérentes visuellement et vérifier l'affichage desktop/mobile.
+Done quand :
+- On a quelque chose de concret : Style homogène
+- La carte est dans la bonne colonne Trello
+Charge : 12 h/h
+Deadline : 18.04.2026</x:v>
       </x:c>
       <x:c r="D17" s="75" t="str">
         <x:v>Jason</x:v>
@@ -4954,11 +4968,12 @@
         <x:v>Finaliser inscription et connexion PHP/MySQL</x:v>
       </x:c>
       <x:c r="C18" s="75" t="str">
-        <x:v>Objectif : Tester la création de compte, la connexion, les erreurs utilisateur et les accès au profil.
-À vérifier :
-- Livrable produit : Auth locale
-- Carte tenue à jour dans la bonne colonne Trello
-Charge : 14 h/h | Échéance : 30.04.2026</x:v>
+        <x:v>Ce qu'on fait : Tester la création de compte, la connexion, les erreurs utilisateur et les accès au profil.
+Done quand :
+- On a quelque chose de concret : Auth locale
+- La carte est dans la bonne colonne Trello
+Charge : 14 h/h
+Deadline : 30.04.2026</x:v>
       </x:c>
       <x:c r="D18" s="75" t="str">
         <x:v>Thierry</x:v>
@@ -4984,11 +4999,12 @@
         <x:v>Configurer OAuth Google et les secrets locaux</x:v>
       </x:c>
       <x:c r="C19" s="75" t="str">
-        <x:v>Objectif : Vérifier le callback Google, remplacer les secrets par des valeurs locales et documenter la configuration.
-À vérifier :
-- Livrable produit : OAuth validé
-- Carte tenue à jour dans la bonne colonne Trello
-Charge : 8 h/h | Échéance : 02.05.2026</x:v>
+        <x:v>Ce qu'on fait : Vérifier le callback Google, remplacer les secrets par des valeurs locales et documenter la configuration.
+Done quand :
+- On a quelque chose de concret : OAuth validé
+- La carte est dans la bonne colonne Trello
+Charge : 8 h/h
+Deadline : 02.05.2026</x:v>
       </x:c>
       <x:c r="D19" s="75" t="str">
         <x:v>Dan</x:v>
@@ -5014,11 +5030,12 @@
         <x:v>Configurer les emails SMTP</x:v>
       </x:c>
       <x:c r="C20" s="75" t="str">
-        <x:v>Objectif : Préparer les variables SMTP, tester les emails liés aux comptes et documenter les paramètres nécessaires.
-À vérifier :
-- Livrable produit : Emails testés
-- Carte tenue à jour dans la bonne colonne Trello
-Charge : 6 h/h | Échéance : 03.05.2026</x:v>
+        <x:v>Ce qu'on fait : Préparer les variables SMTP, tester les emails liés aux comptes et documenter les paramètres nécessaires.
+Done quand :
+- On a quelque chose de concret : Emails testés
+- La carte est dans la bonne colonne Trello
+Charge : 6 h/h
+Deadline : 03.05.2026</x:v>
       </x:c>
       <x:c r="D20" s="75" t="str">
         <x:v>Jason</x:v>
@@ -5044,11 +5061,12 @@
         <x:v>Tester MySQL, phpMyAdmin et l'initialisation SQL</x:v>
       </x:c>
       <x:c r="C21" s="75" t="str">
-        <x:v>Objectif : Vérifier le chargement automatique du schema SQL, l'accès phpMyAdmin et les données nécessaires au site.
-À vérifier :
-- Livrable produit : BDD testée
-- Carte tenue à jour dans la bonne colonne Trello
-Charge : 5 h/h | Échéance : 02.05.2026</x:v>
+        <x:v>Ce qu'on fait : Vérifier le chargement automatique du schema SQL, l'accès phpMyAdmin et les données nécessaires au site.
+Done quand :
+- On a quelque chose de concret : BDD testée
+- La carte est dans la bonne colonne Trello
+Charge : 5 h/h
+Deadline : 02.05.2026</x:v>
       </x:c>
       <x:c r="D21" s="75" t="str">
         <x:v>Dan</x:v>
@@ -5074,12 +5092,13 @@
         <x:v>Mettre à jour Trello et la documentation de séance</x:v>
       </x:c>
       <x:c r="C22" s="75" t="str">
-        <x:v>Objectif : Noter les tâches réalisées, les problèmes, le respect du planning et les adaptations nécessaires.
-À vérifier :
-- Livrable produit : Suivi actualisé
-- Carte tenue à jour dans la bonne colonne Trello
-- Contrôle consigne : Consigne Projet.pdf p.3
-Charge : 8 h/h | Échéance : 05.05.2026</x:v>
+        <x:v>Ce qu'on fait : Noter les tâches réalisées, les problèmes, le respect du planning et les adaptations nécessaires.
+Done quand :
+- On a quelque chose de concret : Suivi actualisé
+- La carte est dans la bonne colonne Trello
+- Ça respecte la consigne : Consigne Projet.pdf p.3
+Charge : 8 h/h
+Deadline : 05.05.2026</x:v>
       </x:c>
       <x:c r="D22" s="75" t="str">
         <x:v>Thierry, Dan, Jason</x:v>
@@ -5105,12 +5124,13 @@
         <x:v>Rendre le Gantt réel actualisé pour l'échéance 2</x:v>
       </x:c>
       <x:c r="C23" s="75" t="str">
-        <x:v>Objectif : Comparer l'avancement réel au prévisionnel et mettre à jour le planning selon les aléas.
-À vérifier :
-- Livrable produit : Gantt réel échéance 2
-- Carte tenue à jour dans la bonne colonne Trello
-- Contrôle consigne : Consigne Projet.pdf p.2-p.3
-Charge : 4 h/h | Échéance : 05.05.2026</x:v>
+        <x:v>Ce qu'on fait : Comparer l'avancement réel au prévisionnel et mettre à jour le planning selon les aléas.
+Done quand :
+- On a quelque chose de concret : Gantt réel échéance 2
+- La carte est dans la bonne colonne Trello
+- Ça respecte la consigne : Consigne Projet.pdf p.2-p.3
+Charge : 4 h/h
+Deadline : 05.05.2026</x:v>
       </x:c>
       <x:c r="D23" s="75" t="str">
         <x:v>Thierry</x:v>
@@ -5136,11 +5156,12 @@
         <x:v>Réaliser les tests fonctionnels complets</x:v>
       </x:c>
       <x:c r="C24" s="75" t="str">
-        <x:v>Objectif : Tester navigation, recherche, pages jeux, inscription, connexion, profil, base de données et erreurs.
-À vérifier :
-- Livrable produit : Plan de tests
-- Carte tenue à jour dans la bonne colonne Trello
-Charge : 10 h/h | Échéance : 14.05.2026</x:v>
+        <x:v>Ce qu'on fait : Tester navigation, recherche, pages jeux, inscription, connexion, profil, base de données et erreurs.
+Done quand :
+- On a quelque chose de concret : Plan de tests
+- La carte est dans la bonne colonne Trello
+Charge : 10 h/h
+Deadline : 14.05.2026</x:v>
       </x:c>
       <x:c r="D24" s="75" t="str">
         <x:v>Thierry, Dan, Jason</x:v>
@@ -5166,11 +5187,12 @@
         <x:v>Corriger les bugs et incohérences de liens</x:v>
       </x:c>
       <x:c r="C25" s="75" t="str">
-        <x:v>Objectif : Corriger les erreurs repérées pendant les tests, notamment chemins, affichage, formulaires et messages.
-À vérifier :
-- Livrable produit : Corrections validées
-- Carte tenue à jour dans la bonne colonne Trello
-Charge : 10 h/h | Échéance : 18.05.2026</x:v>
+        <x:v>Ce qu'on fait : Corriger les erreurs repérées pendant les tests, notamment chemins, affichage, formulaires et messages.
+Done quand :
+- On a quelque chose de concret : Corrections validées
+- La carte est dans la bonne colonne Trello
+Charge : 10 h/h
+Deadline : 18.05.2026</x:v>
       </x:c>
       <x:c r="D25" s="75" t="str">
         <x:v>Thierry, Dan, Jason</x:v>
@@ -5196,11 +5218,12 @@
         <x:v>Sécuriser la configuration et nettoyer les secrets</x:v>
       </x:c>
       <x:c r="C26" s="75" t="str">
-        <x:v>Objectif : Vérifier que les secrets OAuth/SMTP ne sont pas exposés et documenter les valeurs à configurer localement.
-À vérifier :
-- Livrable produit : Config propre
-- Carte tenue à jour dans la bonne colonne Trello
-Charge : 6 h/h | Échéance : 15.05.2026</x:v>
+        <x:v>Ce qu'on fait : Vérifier que les secrets OAuth/SMTP ne sont pas exposés et documenter les valeurs à configurer localement.
+Done quand :
+- On a quelque chose de concret : Config propre
+- La carte est dans la bonne colonne Trello
+Charge : 6 h/h
+Deadline : 15.05.2026</x:v>
       </x:c>
       <x:c r="D26" s="75" t="str">
         <x:v>Dan</x:v>
@@ -5226,12 +5249,13 @@
         <x:v>Préparer Docker final et README de lancement</x:v>
       </x:c>
       <x:c r="C27" s="75" t="str">
-        <x:v>Objectif : Vérifier que docker compose lance toute l'application et que le README explique les URLs et commandes.
-À vérifier :
-- Livrable produit : README final
-- Carte tenue à jour dans la bonne colonne Trello
-- Contrôle consigne : Consigne Projet.pdf p.4
-Charge : 6 h/h | Échéance : 19.05.2026</x:v>
+        <x:v>Ce qu'on fait : Vérifier que docker compose lance toute l'application et que le README explique les URLs et commandes.
+Done quand :
+- On a quelque chose de concret : README final
+- La carte est dans la bonne colonne Trello
+- Ça respecte la consigne : Consigne Projet.pdf p.4
+Charge : 6 h/h
+Deadline : 19.05.2026</x:v>
       </x:c>
       <x:c r="D27" s="75" t="str">
         <x:v>Thierry</x:v>
@@ -5257,12 +5281,13 @@
         <x:v>Finaliser la documentation et la synthèse de clôture</x:v>
       </x:c>
       <x:c r="C28" s="75" t="str">
-        <x:v>Objectif : Ajouter ressenti du groupe, écarts de planning, tâches non terminées et impact de la gestion de projet.
-À vérifier :
-- Livrable produit : Document final
-- Carte tenue à jour dans la bonne colonne Trello
-- Contrôle consigne : Consigne Projet.pdf p.4
-Charge : 10 h/h | Échéance : 26.05.2026</x:v>
+        <x:v>Ce qu'on fait : Ajouter ressenti du groupe, écarts de planning, tâches non terminées et impact de la gestion de projet.
+Done quand :
+- On a quelque chose de concret : Document final
+- La carte est dans la bonne colonne Trello
+- Ça respecte la consigne : Consigne Projet.pdf p.4
+Charge : 10 h/h
+Deadline : 26.05.2026</x:v>
       </x:c>
       <x:c r="D28" s="75" t="str">
         <x:v>Jason</x:v>
@@ -5288,12 +5313,13 @@
         <x:v>Produire le Gantt réel final et comparer avec l'initial</x:v>
       </x:c>
       <x:c r="C29" s="75" t="str">
-        <x:v>Objectif : Renseigner les dates réelles, les écarts et expliquer les adaptations du planning.
-À vérifier :
-- Livrable produit : Gantt réel final
-- Carte tenue à jour dans la bonne colonne Trello
-- Contrôle consigne : Consigne Projet.pdf p.3-p.4
-Charge : 4 h/h | Échéance : 26.05.2026</x:v>
+        <x:v>Ce qu'on fait : Renseigner les dates réelles, les écarts et expliquer les adaptations du planning.
+Done quand :
+- On a quelque chose de concret : Gantt réel final
+- La carte est dans la bonne colonne Trello
+- Ça respecte la consigne : Consigne Projet.pdf p.3-p.4
+Charge : 4 h/h
+Deadline : 26.05.2026</x:v>
       </x:c>
       <x:c r="D29" s="75" t="str">
         <x:v>Thierry</x:v>
@@ -5319,12 +5345,13 @@
         <x:v>Créer le support de présentation</x:v>
       </x:c>
       <x:c r="C30" s="75" t="str">
-        <x:v>Objectif : Préparer les diapositives sur projet, équipe, planning initial/final, outils, réalisation et ressenti.
-À vérifier :
-- Livrable produit : Slides numérotées
-- Carte tenue à jour dans la bonne colonne Trello
-- Contrôle consigne : Consigne Projet.pdf p.4
-Charge : 8 h/h | Échéance : 08.06.2026</x:v>
+        <x:v>Ce qu'on fait : Préparer les diapositives sur projet, équipe, planning initial/final, outils, réalisation et ressenti.
+Done quand :
+- On a quelque chose de concret : Slides numérotées
+- La carte est dans la bonne colonne Trello
+- Ça respecte la consigne : Consigne Projet.pdf p.4
+Charge : 8 h/h
+Deadline : 08.06.2026</x:v>
       </x:c>
       <x:c r="D30" s="75" t="str">
         <x:v>Thierry, Dan, Jason</x:v>
@@ -5350,12 +5377,13 @@
         <x:v>Répéter et répartir le temps de parole</x:v>
       </x:c>
       <x:c r="C31" s="78" t="str">
-        <x:v>Objectif : Préparer une présentation de 10 minutes avec un temps de parole équivalent pour chaque membre.
-À vérifier :
-- Livrable produit : Répétition prête
-- Carte tenue à jour dans la bonne colonne Trello
-- Contrôle consigne : Consigne Projet.pdf p.4
-Charge : 4 h/h | Échéance : 08.06.2026</x:v>
+        <x:v>Ce qu'on fait : Préparer une présentation de 10 minutes avec un temps de parole équivalent pour chaque membre.
+Done quand :
+- On a quelque chose de concret : Répétition prête
+- La carte est dans la bonne colonne Trello
+- Ça respecte la consigne : Consigne Projet.pdf p.4
+Charge : 4 h/h
+Deadline : 08.06.2026</x:v>
       </x:c>
       <x:c r="D31" s="78" t="str">
         <x:v>Thierry, Dan, Jason</x:v>
@@ -5384,7 +5412,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rcfc4f9f572c3404e"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R26f32ed99c314fe7"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5718,7 +5746,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb7f0167958fa42a3"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4c64be4e944a43e2"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>